<commit_message>
📊 Horarios actualizados Línea 141 - 1611
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:06:31</t>
+          <t>Última actualización: 02:42:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:06:31</t>
+          <t>02:42:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:25</t>
+          <t>03:03</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,23 +498,48 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:06:31</t>
+          <t>02:42:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>116</v>
+        <v>66</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:42:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>04:02</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -544,7 +569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:06:31</t>
+          <t>Última actualización: 02:42:00</t>
         </is>
       </c>
     </row>
@@ -579,7 +604,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:06:31</t>
+          <t>Última actualización: 02:42:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1612
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:42:00</t>
+          <t>Última actualización: 03:38:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:42:00</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:03</t>
+          <t>03:47</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:42:00</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>03:50</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>83_ESC 6_ALUAR</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,23 +523,198 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:42:00</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:02</t>
+          <t>04:31</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>80</v>
+        <v>53</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>03:38:59</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:47</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>69</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>03:38:59</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>70</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>03:38:59</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>05:06</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>88</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>03:38:59</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>05:19</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>101</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>03:38:59</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>05:28</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>110</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>03:38:59</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>05:28</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>110</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>03:38:59</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>112</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -556,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,14 +744,91 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:42:00</t>
+          <t>Última actualización: 03:38:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>03:38:59</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>70</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>03:38:59</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>05:28</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>110</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -591,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -604,14 +856,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:42:00</t>
+          <t>Última actualización: 03:38:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>03:38:59</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>05:28</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>110</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1613
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:38:59</t>
+          <t>Última actualización: 04:30:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>04:36</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>69</v>
+        <v>6</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>70</v>
+        <v>17</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -603,16 +603,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:06</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -628,16 +628,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>05:19</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>101</v>
+        <v>70</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>05:28</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>110</v>
+        <v>23</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -678,16 +678,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>05:28</t>
+          <t>05:06</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -703,18 +703,268 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>05:19</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>101</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:30:32</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>05:22</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>52</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>03:38:59</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>05:28</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>110</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>03:38:59</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>05:28</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>110</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>03:38:59</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>05:30</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D19" t="n">
         <v>112</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>04:30:32</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>05:44</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>74</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>04:30:32</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>05:47</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>77</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>04:30:32</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>91</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>04:30:32</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>06:09</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>99</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>04:30:32</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>102</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>04:30:32</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>06:27</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>117</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -731,7 +981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -744,14 +994,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:38:59</t>
+          <t>Última actualización: 04:30:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -827,6 +1077,31 @@
         <v>110</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>04:30:32</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>102</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -856,7 +1131,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:38:59</t>
+          <t>Última actualización: 04:30:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1614
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:30:32</t>
+          <t>Última actualización: 05:01:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -583,11 +583,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -608,11 +608,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -673,12 +673,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>05:01:17</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>05:06</t>
+          <t>05:02</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>88</v>
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -703,16 +703,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>05:19</t>
+          <t>05:06</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:19</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>52</v>
+        <v>101</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,12 +748,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>05:01:17</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>05:28</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>110</v>
+        <v>21</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -803,16 +803,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>05:30</t>
+          <t>05:28</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>05:30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>74</v>
+        <v>112</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>05:01:17</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,21 +873,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>05:01:17</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>91</v>
+        <v>46</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>05:01:17</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>99</v>
+        <v>60</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,21 +923,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>05:01:17</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>102</v>
+        <v>68</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,23 +948,223 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>05:01:17</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>71</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>04:30:32</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>06:27</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="D26" t="n">
         <v>117</v>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>05:01:17</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>89</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>05:01:17</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>06:34</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>93</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>05:01:17</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>98</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>05:01:17</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>100</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>05:01:17</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>06:45</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>104</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>05:01:17</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>114</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>05:01:17</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>06:59</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>118</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -981,7 +1181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -994,14 +1194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:30:32</t>
+          <t>Última actualización: 05:01:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1285,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>05:01:17</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1099,9 +1299,34 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>102</v>
+        <v>71</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>05:01:17</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>114</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1131,7 +1356,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:30:32</t>
+          <t>Última actualización: 05:01:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1615
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:01:17</t>
+          <t>Última actualización: 05:51:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>05:01:17</t>
+          <t>05:51:39</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>05:01:17</t>
+          <t>05:51:39</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,7 +948,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>05:01:17</t>
+          <t>05:51:39</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>05:01:17</t>
+          <t>05:51:39</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>89</v>
+        <v>39</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>05:01:17</t>
+          <t>05:51:39</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>05:01:17</t>
+          <t>05:51:39</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>98</v>
+        <v>48</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,12 +1073,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>05:01:17</t>
+          <t>05:51:39</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1103,16 +1103,16 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>06:45</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1128,16 +1128,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>06:55</t>
+          <t>06:45</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,23 +1148,198 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>05:01:17</t>
+          <t>05:51:39</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>64</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>05:51:39</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>06:59</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>118</v>
-      </c>
-      <c r="E33" t="inlineStr">
+      <c r="D34" t="n">
+        <v>68</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>05:51:39</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>07:19</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>88</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>05:51:39</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>07:19</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>88</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>05:51:39</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>100</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>05:51:39</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>104</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>05:51:39</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>105</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>05:51:39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>07:39</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>108</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1181,7 +1356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1194,14 +1369,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:01:17</t>
+          <t>Última actualización: 05:51:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1460,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:01:17</t>
+          <t>05:51:39</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1299,7 +1474,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1310,7 +1485,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:01:17</t>
+          <t>05:51:39</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1324,9 +1499,34 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>114</v>
+        <v>64</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>05:51:39</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>07:19</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>88</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1343,7 +1543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1356,14 +1556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:01:17</t>
+          <t>Última actualización: 05:51:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -1416,6 +1616,31 @@
       <c r="E6" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:51:39</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:43</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>112</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1616
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:51:39</t>
+          <t>Última actualización: 06:23:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -583,11 +583,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -608,11 +608,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>05:51:39</t>
+          <t>06:23:30</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>05:51:39</t>
+          <t>06:23:30</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>05:51:39</t>
+          <t>06:23:30</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:01:17</t>
+          <t>06:23:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>100</v>
+        <v>18</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1148,21 +1148,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>05:51:39</t>
+          <t>06:23:30</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>06:55</t>
+          <t>06:49</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>05:51:39</t>
+          <t>06:23:30</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>05:51:39</t>
+          <t>06:23:30</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>88</v>
+        <v>36</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,7 +1223,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>05:51:39</t>
+          <t>06:23:30</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>88</v>
+        <v>56</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>05:51:39</t>
+          <t>06:23:30</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1278,16 +1278,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>05:51:39</t>
+          <t>06:23:30</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>105</v>
+        <v>71</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,23 +1323,223 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>06:23:30</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>07:34</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>71</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>06:23:30</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>72</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>06:23:30</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>73</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>05:51:39</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>07:39</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D40" t="n">
+      <c r="D43" t="n">
         <v>108</v>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>06:23:30</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>92</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>06:23:30</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>97</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>06:23:30</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>98</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>06:23:30</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>08:11</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>108</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>06:23:30</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>08:17</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>114</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1356,7 +1556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1369,14 +1569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:51:39</t>
+          <t>Última actualización: 06:23:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1685,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:51:39</t>
+          <t>06:23:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1499,7 +1699,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1510,7 +1710,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:51:39</t>
+          <t>06:23:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1524,9 +1724,34 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>88</v>
+        <v>56</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06:23:30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>07:34</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>71</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1543,7 +1768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1556,14 +1781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:51:39</t>
+          <t>Última actualización: 06:23:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -1639,6 +1864,31 @@
         <v>112</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:23:30</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>81</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1617
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:23:30</t>
+          <t>Última actualización: 06:54:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 52</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,21 +1223,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>56</v>
+        <v>5</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>05:51:39</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>05:51:39</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>07:34</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>71</v>
+        <v>100</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>73</v>
+        <v>41</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>05:51:39</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>07:39</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>108</v>
+        <v>42</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,12 +1423,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>05:51:39</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:39</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:42</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>97</v>
+        <v>48</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>98</v>
+        <v>61</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>108</v>
+        <v>65</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1528,18 +1528,243 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>97</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>06:54:35</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>67</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>06:23:30</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>08:11</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>108</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>06:54:35</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
           <t>08:17</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D48" t="n">
-        <v>114</v>
-      </c>
-      <c r="E48" t="inlineStr">
+      <c r="D51" t="n">
+        <v>83</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>06:54:35</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>87</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>06:54:35</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>08:26</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>92</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>06:54:35</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>08:28</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>94</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>06:54:35</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>104</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>06:54:35</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>107</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>06:54:35</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>107</v>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1556,7 +1781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1569,14 +1794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:23:30</t>
+          <t>Última actualización: 06:54:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1910,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1699,7 +1924,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1710,7 +1935,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1724,7 +1949,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1735,7 +1960,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1749,9 +1974,34 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>71</v>
+        <v>40</v>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>06:54:35</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>104</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1768,7 +2018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1781,14 +2031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:23:30</t>
+          <t>Última actualización: 06:54:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1872,7 +2122,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1886,11 +2136,61 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>81</v>
+        <v>50</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:54:35</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>99</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06:54:35</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:47</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>113</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1618
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:54:35</t>
+          <t>Última actualización: 07:18:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 52</t>
+          <t>Total filas: 59</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -583,11 +583,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -608,11 +608,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>05:51:39</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>07:34</t>
+          <t>07:24</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>71</v>
+        <v>6</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>05:51:39</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>07:34</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>05:51:39</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>07:39</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>108</v>
+        <v>17</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>07:42</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>48</v>
+        <v>18</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,12 +1473,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>05:51:39</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:39</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>61</v>
+        <v>108</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1503,16 +1503,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:42</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1578,16 +1578,16 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>08:17</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>83</v>
+        <v>43</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>06:23:30</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:11</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>08:26</t>
+          <t>08:17</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>92</v>
+        <v>59</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>08:28</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>94</v>
+        <v>63</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1703,16 +1703,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>08:38</t>
+          <t>08:26</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:28</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>107</v>
+        <v>70</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,23 +1748,198 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>80</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>07:18:31</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
           <t>08:41</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D57" t="n">
-        <v>107</v>
-      </c>
-      <c r="E57" t="inlineStr">
+      <c r="D58" t="n">
+        <v>83</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>07:18:31</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>83</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>07:18:31</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>08:50</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>92</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>07:18:31</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>96</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>07:18:31</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>98</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>07:18:31</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>118</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>07:18:31</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>119</v>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1781,7 +1956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1794,14 +1969,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:54:35</t>
+          <t>Última actualización: 07:18:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1935,7 +2110,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1949,7 +2124,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1960,7 +2135,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1974,7 +2149,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1985,7 +2160,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1999,9 +2174,59 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07:18:31</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>96</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>07:18:31</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>98</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2018,7 +2243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2031,14 +2256,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:54:35</t>
+          <t>Última actualización: 07:18:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2347,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2136,7 +2361,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2147,7 +2372,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2161,7 +2386,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2189,6 +2414,31 @@
         <v>113</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07:18:31</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>90</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1619
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:18:31</t>
+          <t>Última actualización: 07:51:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 59</t>
+          <t>Total filas: 66</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,7 +1623,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>06:23:30</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1637,7 +1637,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>108</v>
+        <v>20</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,7 +1648,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1662,7 +1662,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>59</v>
+        <v>26</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>63</v>
+        <v>30</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>70</v>
+        <v>37</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>80</v>
+        <v>47</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>83</v>
+        <v>50</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1812,7 +1812,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>83</v>
+        <v>50</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>96</v>
+        <v>63</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>98</v>
+        <v>65</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>118</v>
+        <v>75</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1928,18 +1928,193 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>118</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>07:51:30</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
           <t>09:17</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>86</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>07:51:30</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
         <is>
           <t>17X38_ROMERO</t>
         </is>
       </c>
-      <c r="D64" t="n">
-        <v>119</v>
-      </c>
-      <c r="E64" t="inlineStr">
+      <c r="D66" t="n">
+        <v>86</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>07:51:30</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>89</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>07:51:30</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>09:26</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>95</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>07:51:30</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>09:38</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>107</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>07:51:30</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>09:41</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>110</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>07:51:30</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>09:43</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>112</v>
+      </c>
+      <c r="E71" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1969,7 +2144,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:18:31</t>
+          <t>Última actualización: 07:51:30</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2335,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2174,7 +2349,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>80</v>
+        <v>47</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2185,7 +2360,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2199,7 +2374,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>96</v>
+        <v>63</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2210,7 +2385,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2224,7 +2399,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>98</v>
+        <v>65</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2243,7 +2418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2256,14 +2431,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:18:31</t>
+          <t>Última actualización: 07:51:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -2372,7 +2547,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2386,7 +2561,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2422,7 +2597,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2436,11 +2611,36 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>90</v>
+        <v>57</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:51:30</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>97</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1620
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:51:30</t>
+          <t>Última actualización: 08:16:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 66</t>
+          <t>Total filas: 73</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -583,11 +583,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -608,11 +608,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1648,7 +1648,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1662,7 +1662,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:57</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>75</v>
+        <v>41</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>118</v>
+        <v>50</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>86</v>
+        <v>118</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>09:20</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>95</v>
+        <v>61</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2053,16 +2053,16 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:20</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>110</v>
+        <v>70</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,23 +2098,198 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
+          <t>09:38</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>82</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>08:16:18</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>09:41</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>85</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>08:16:18</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
           <t>09:43</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D71" t="n">
+      <c r="D73" t="n">
+        <v>87</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>08:16:18</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>100</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>08:16:18</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>102</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>08:16:18</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>102</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>08:16:18</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>10:08</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
         <v>112</v>
       </c>
-      <c r="E71" t="inlineStr">
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>08:16:18</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>117</v>
+      </c>
+      <c r="E78" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2131,7 +2306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2144,14 +2319,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:51:30</t>
+          <t>Última actualización: 08:16:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2510,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2349,7 +2524,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2360,7 +2535,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2374,7 +2549,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2402,6 +2577,56 @@
         <v>65</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:16:18</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>08:57</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>41</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08:16:18</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>102</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2418,7 +2643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2431,14 +2656,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:51:30</t>
+          <t>Última actualización: 08:16:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -2547,7 +2772,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2561,7 +2786,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2597,7 +2822,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2611,7 +2836,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>57</v>
+        <v>32</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2622,7 +2847,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2636,11 +2861,36 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>97</v>
+        <v>72</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:16:18</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>10:08</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>112</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1621
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:16:18</t>
+          <t>Última actualización: 08:41:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 73</t>
+          <t>Total filas: 82</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -583,11 +583,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -608,11 +608,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1812,7 +1812,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>65</v>
+        <v>15</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>118</v>
+        <v>30</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2003,16 +2003,16 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,12 +2023,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>09:20</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>07:51:30</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:20</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>85</v>
+        <v>45</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>09:43</t>
+          <t>09:31</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>87</v>
+        <v>50</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:38</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>100</v>
+        <v>57</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>09:43</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>102</v>
+        <v>62</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>10:08</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>112</v>
+        <v>74</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,23 +2273,248 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
+          <t>08:41:47</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>75</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>08:41:47</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>76</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
           <t>08:16:18</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>102</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>08:16:18</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>102</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>08:41:47</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>09:59</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>78</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>08:16:18</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>10:08</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>112</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>08:41:47</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>10:09</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>88</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>08:41:47</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
         <is>
           <t>10:13</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D78" t="n">
-        <v>117</v>
-      </c>
-      <c r="E78" t="inlineStr">
+      <c r="D85" t="n">
+        <v>92</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>08:41:47</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>105</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>08:41:47</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>106</v>
+      </c>
+      <c r="E87" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2306,7 +2531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2319,14 +2544,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:16:18</t>
+          <t>Última actualización: 08:41:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2760,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2549,7 +2774,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2560,7 +2785,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:51:30</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2574,7 +2799,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>65</v>
+        <v>15</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2610,23 +2835,48 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>08:41:47</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>76</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>08:16:18</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>09:58</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D17" t="n">
         <v>102</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2643,7 +2893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2656,14 +2906,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:16:18</t>
+          <t>Última actualización: 08:41:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2797,7 +3047,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2811,7 +3061,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>113</v>
+        <v>6</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2847,12 +3097,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>09:28</t>
+          <t>09:27</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2861,7 +3111,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2877,20 +3127,120 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>72</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:41:47</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>86</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:16:18</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>10:08</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D15" t="n">
         <v>112</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08:41:47</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>106</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:41:47</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>113</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1622
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:E92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:41:47</t>
+          <t>Última actualización: 08:57:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 82</t>
+          <t>Total filas: 87</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1912,7 +1912,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>50</v>
+        <v>9</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2123,7 +2123,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2187,7 +2187,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2212,7 +2212,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>09:57</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2373,21 +2373,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>09:59</t>
+          <t>09:58</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>10:08</t>
+          <t>09:59</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>112</v>
+        <v>78</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,12 +2423,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>10:09</t>
+          <t>10:08</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2453,16 +2453,16 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>10:13</t>
+          <t>10:09</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:11</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>105</v>
+        <v>74</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2503,18 +2503,143 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>92</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>08:57:38</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>78</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>08:57:38</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>89</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>08:57:38</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
           <t>10:27</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C90" t="inlineStr">
         <is>
           <t>17X38_ROMERO</t>
         </is>
       </c>
-      <c r="D87" t="n">
+      <c r="D90" t="n">
+        <v>90</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>08:57:38</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
         <v>106</v>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>08:57:38</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>107</v>
+      </c>
+      <c r="E92" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2544,7 +2669,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:41:47</t>
+          <t>Última actualización: 08:57:38</t>
         </is>
       </c>
     </row>
@@ -2810,7 +2935,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2824,7 +2949,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2835,7 +2960,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2849,7 +2974,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2893,7 +3018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2906,14 +3031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:41:47</t>
+          <t>Última actualización: 08:57:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -3097,7 +3222,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3111,7 +3236,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -3147,7 +3272,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3161,7 +3286,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -3197,7 +3322,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3211,7 +3336,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3239,6 +3364,31 @@
         <v>113</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:57:38</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>98</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1623
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E92"/>
+  <dimension ref="A1:E104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:57:38</t>
+          <t>Última actualización: 09:40:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 87</t>
+          <t>Total filas: 99</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>10:08</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>112</v>
+        <v>21</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>10:09</t>
+          <t>10:05</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>88</v>
+        <v>25</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,12 +2473,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>10:08</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2487,7 +2487,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>74</v>
+        <v>112</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2503,16 +2503,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>10:13</t>
+          <t>10:09</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>10:11</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>78</v>
+        <v>31</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:13</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>89</v>
+        <v>33</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2578,16 +2578,16 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>10:27</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>106</v>
+        <v>46</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,23 +2623,323 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>47</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>63</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
           <t>10:44</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
+      <c r="C94" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D92" t="n">
-        <v>107</v>
-      </c>
-      <c r="E92" t="inlineStr">
+      <c r="D94" t="n">
+        <v>64</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>10:52</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>72</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>75</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>75</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>78</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>82</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>90</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>93</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>108</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>114</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>118</v>
+      </c>
+      <c r="E104" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2656,7 +2956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2669,14 +2969,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:57:38</t>
+          <t>Última actualización: 09:40:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2985,7 +3285,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2999,9 +3299,59 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>108</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>118</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3018,7 +3368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3031,14 +3381,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:57:38</t>
+          <t>Última actualización: 09:40:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3647,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3311,7 +3661,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>112</v>
+        <v>28</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -3347,21 +3697,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:28</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>113</v>
+        <v>48</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3372,25 +3722,75 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>113</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>10:35</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>98</v>
-      </c>
-      <c r="E18" t="inlineStr">
+      <c r="D19" t="n">
+        <v>55</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>108</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1624
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E104"/>
+  <dimension ref="A1:E116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:40:26</t>
+          <t>Última actualización: 10:35:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 99</t>
+          <t>Total filas: 111</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2648,7 +2648,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2662,7 +2662,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>63</v>
+        <v>8</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>64</v>
+        <v>9</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>10:55</t>
+          <t>10:52</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>75</v>
+        <v>17</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2778,16 +2778,16 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>10:58</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>11:02</t>
+          <t>10:56</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>82</v>
+        <v>21</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>10:58</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>90</v>
+        <v>23</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,21 +2848,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>11:13</t>
+          <t>11:02</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>93</v>
+        <v>27</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>11:28</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>108</v>
+        <v>35</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>11:34</t>
+          <t>11:13</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,23 +2923,323 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
+          <t>10:35:48</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>45</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>10:35:48</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>50</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>10:35:48</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>52</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
           <t>09:40:26</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr">
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>108</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>09:40:26</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>114</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>10:35:48</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
         <is>
           <t>11:38</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr">
+      <c r="C109" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D104" t="n">
-        <v>118</v>
-      </c>
-      <c r="E104" t="inlineStr">
+      <c r="D109" t="n">
+        <v>63</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>10:35:48</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>67</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>10:35:48</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>67</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>10:35:48</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>11:53</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>78</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>10:35:48</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>83</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>10:35:48</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>93</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>10:35:48</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>12:13</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>98</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>10:35:48</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>112</v>
+      </c>
+      <c r="E116" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2956,7 +3256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2969,14 +3269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:40:26</t>
+          <t>Última actualización: 10:35:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3310,12 +3610,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11:28</t>
+          <t>11:27</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3324,7 +3624,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>108</v>
+        <v>52</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3340,18 +3640,68 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>108</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10:35:48</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>11:38</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>118</v>
-      </c>
-      <c r="E19" t="inlineStr">
+      <c r="D20" t="n">
+        <v>63</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10:35:48</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>112</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3368,7 +3718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3381,14 +3731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:40:26</t>
+          <t>Última actualización: 10:35:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3747,7 +4097,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3761,7 +4111,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3772,23 +4122,48 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>10:35:48</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>52</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>09:40:26</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>11:28</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D20" t="n">
+      <c r="D21" t="n">
         <v>108</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1625
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E116"/>
+  <dimension ref="A1:E125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:35:48</t>
+          <t>Última actualización: 11:04:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 111</t>
+          <t>Total filas: 120</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2912,7 +2912,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2962,7 +2962,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3012,7 +3012,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3062,7 +3062,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>11:42</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:42</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>83</v>
+        <v>49</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>12:13</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>98</v>
+        <v>54</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,23 +3223,248 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
+          <t>11:04:33</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>64</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>11:04:33</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>12:13</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>69</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>11:04:33</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>12:23</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>79</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
           <t>10:35:48</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr">
+      <c r="B119" t="inlineStr">
         <is>
           <t>12:27</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
+      <c r="C119" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D116" t="n">
+      <c r="D119" t="n">
         <v>112</v>
       </c>
-      <c r="E116" t="inlineStr">
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>11:04:33</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>84</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>11:04:33</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>88</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>11:04:33</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>94</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>11:04:33</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>96</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>11:04:33</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>12:42</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>98</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>11:04:33</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>112</v>
+      </c>
+      <c r="E125" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3256,7 +3481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3269,14 +3494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:35:48</t>
+          <t>Última actualización: 11:04:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3635,7 +3860,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3649,7 +3874,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3660,7 +3885,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3674,7 +3899,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3702,6 +3927,31 @@
         <v>112</v>
       </c>
       <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>11:04:33</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>84</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3718,7 +3968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3731,14 +3981,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:35:48</t>
+          <t>Última actualización: 11:04:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4397,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4161,9 +4411,34 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="E21" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>11:04:33</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>114</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1626
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E125"/>
+  <dimension ref="A1:E140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:04:33</t>
+          <t>Última actualización: 11:43:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 120</t>
+          <t>Total filas: 135</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>64</v>
+        <v>15</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3253,16 +3253,16 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>12:13</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:09</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>79</v>
+        <v>26</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>112</v>
+        <v>27</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:13</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>84</v>
+        <v>30</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3353,16 +3353,16 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:27</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>12:40</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>96</v>
+        <v>45</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>12:42</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>98</v>
+        <v>48</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3453,18 +3453,393 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>88</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>12:37</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>54</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>11:04:33</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>94</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>12:39</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>56</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>11:04:33</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>96</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>12:42</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>59</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>11:04:33</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
           <t>12:56</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr">
+      <c r="C131" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D125" t="n">
+      <c r="D131" t="n">
         <v>112</v>
       </c>
-      <c r="E125" t="inlineStr">
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>74</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>75</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>90</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>13:14</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>91</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>98</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>101</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>105</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>110</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>117</v>
+      </c>
+      <c r="E140" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3481,7 +3856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3494,14 +3869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:04:33</t>
+          <t>Última actualización: 11:43:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3935,7 +4310,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3949,9 +4324,59 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>84</v>
+        <v>45</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>75</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>101</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3968,7 +4393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3981,14 +4406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:04:33</t>
+          <t>Última actualización: 11:43:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4847,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4436,11 +4861,36 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>114</v>
+        <v>75</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:29</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>106</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1627
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E140"/>
+  <dimension ref="A1:E146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:43:13</t>
+          <t>Última actualización: 12:02:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 135</t>
+          <t>Total filas: 141</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -583,11 +583,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -608,11 +608,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3262,7 +3262,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3298,7 +3298,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3337,7 +3337,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3362,7 +3362,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>79</v>
+        <v>21</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3412,7 +3412,7 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3473,12 +3473,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -3487,7 +3487,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>94</v>
+        <v>54</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,12 +3523,12 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>12:39</t>
+          <t>12:38</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3537,7 +3537,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>12:40</t>
+          <t>12:39</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>96</v>
+        <v>56</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>12:42</t>
+          <t>12:40</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>59</v>
+        <v>96</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:42</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>112</v>
+        <v>40</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>12:58</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3678,16 +3678,16 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>91</v>
+        <v>56</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>98</v>
+        <v>71</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>101</v>
+        <v>72</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3778,16 +3778,16 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>13:28</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>110</v>
+        <v>82</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,23 +3823,173 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
+          <t>12:02:25</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>83</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
           <t>11:43:13</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr">
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>105</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>12:02:25</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>90</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>11:43:13</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>110</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>12:02:25</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
         <is>
           <t>13:40</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr">
+      <c r="C144" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D140" t="n">
-        <v>117</v>
-      </c>
-      <c r="E140" t="inlineStr">
+      <c r="D144" t="n">
+        <v>98</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>12:02:25</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>105</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>12:02:25</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>108</v>
+      </c>
+      <c r="E146" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3869,7 +4019,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:43:13</t>
+          <t>Última actualización: 12:02:25</t>
         </is>
       </c>
     </row>
@@ -4310,7 +4460,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4324,7 +4474,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -4335,7 +4485,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4349,7 +4499,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4360,7 +4510,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4374,7 +4524,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4393,7 +4543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4406,14 +4556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:43:13</t>
+          <t>Última actualización: 12:02:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -4847,7 +4997,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4861,7 +5011,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -4872,7 +5022,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4886,11 +5036,36 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>12:02:25</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:53</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>111</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1628
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E146"/>
+  <dimension ref="A1:E153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:02:25</t>
+          <t>Última actualización: 12:39:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 141</t>
+          <t>Total filas: 148</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>12:40</t>
+          <t>12:39</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>12:42</t>
+          <t>12:40</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>40</v>
+        <v>96</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:42</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>53</v>
+        <v>3</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,12 +3673,12 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -3687,7 +3687,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>74</v>
+        <v>17</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>12:58</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>71</v>
+        <v>19</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>72</v>
+        <v>34</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>98</v>
+        <v>35</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>82</v>
+        <v>42</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>83</v>
+        <v>45</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>13:28</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>105</v>
+        <v>83</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:28</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,12 +3898,12 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>110</v>
+        <v>53</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:40</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>105</v>
+        <v>61</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,23 +3973,198 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>68</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>12:39:18</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
           <t>13:50</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr">
+      <c r="C147" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D146" t="n">
-        <v>108</v>
-      </c>
-      <c r="E146" t="inlineStr">
+      <c r="D147" t="n">
+        <v>71</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>12:39:18</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>14:08</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>89</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>12:39:18</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>14:08</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>89</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>12:39:18</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>92</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>12:39:18</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>98</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>12:39:18</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>107</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>12:39:18</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>109</v>
+      </c>
+      <c r="E153" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4006,7 +4181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4019,14 +4194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:02:25</t>
+          <t>Última actualización: 12:39:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -4485,7 +4660,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4499,7 +4674,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4510,7 +4685,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4524,9 +4699,34 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>12:39:18</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>109</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4556,7 +4756,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:02:25</t>
+          <t>Última actualización: 12:39:18</t>
         </is>
       </c>
     </row>
@@ -4997,7 +5197,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -5011,7 +5211,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -5022,7 +5222,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5036,7 +5236,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>87</v>
+        <v>50</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -5047,7 +5247,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5061,7 +5261,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>111</v>
+        <v>74</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1629
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E153"/>
+  <dimension ref="A1:E163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:39:18</t>
+          <t>Última actualización: 12:56:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 148</t>
+          <t>Total filas: 158</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -583,11 +583,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -608,11 +608,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,12 +3698,12 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -3712,7 +3712,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,12 +3723,12 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>12:58</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3778,16 +3778,16 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>12:02:25</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>83</v>
+        <v>35</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>13:28</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>105</v>
+        <v>25</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:02:25</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>110</v>
+        <v>83</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>13:28</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>61</v>
+        <v>105</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>71</v>
+        <v>110</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>13:40</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>89</v>
+        <v>51</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>13:49</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>92</v>
+        <v>53</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4103,16 +4103,16 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>98</v>
+        <v>71</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:07</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>107</v>
+        <v>71</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,23 +4148,273 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
+          <t>12:56:54</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>14:08</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>72</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
           <t>12:39:18</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr">
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>14:08</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>89</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>12:56:54</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>75</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>12:56:54</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>80</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>12:39:18</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>98</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>12:56:54</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>90</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>12:56:54</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>91</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>12:39:18</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
         <is>
           <t>14:28</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr">
+      <c r="C160" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D153" t="n">
+      <c r="D160" t="n">
         <v>109</v>
       </c>
-      <c r="E153" t="inlineStr">
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>12:56:54</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>104</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>12:56:54</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>111</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>12:56:54</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>119</v>
+      </c>
+      <c r="E163" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4181,7 +4431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4194,14 +4444,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:39:18</t>
+          <t>Última actualización: 12:56:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -4660,12 +4910,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>12:58</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -4674,7 +4924,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4690,16 +4940,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4710,23 +4960,98 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>12:56:54</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>28</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>12:56:54</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>91</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>12:39:18</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>14:28</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="D27" t="n">
         <v>109</v>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>12:56:54</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>111</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4743,7 +5068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4756,14 +5081,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:39:18</t>
+          <t>Última actualización: 12:56:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -5222,48 +5547,123 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>13:29</t>
+          <t>12:59</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>12:56:54</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>32</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>12:39:18</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>13:29</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>50</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>12:56:54</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>13:52</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>56</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>12:39:18</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>13:53</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D27" t="n">
         <v>74</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1630
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E163"/>
+  <dimension ref="A1:E170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:56:54</t>
+          <t>Última actualización: 13:23:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 158</t>
+          <t>Total filas: 165</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>38</v>
+        <v>67</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4037,7 +4037,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4062,7 +4062,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4112,7 +4112,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>72</v>
+        <v>45</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4183,11 +4183,11 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4212,7 +4212,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>75</v>
+        <v>48</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>80</v>
+        <v>53</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:26</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,12 +4323,12 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>109</v>
+        <v>64</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4378,16 +4378,16 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,23 +4398,198 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>78</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>13:23:42</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>84</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>13:23:42</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
           <t>14:55</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr">
+      <c r="C165" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D163" t="n">
-        <v>119</v>
-      </c>
-      <c r="E163" t="inlineStr">
+      <c r="D165" t="n">
+        <v>92</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>13:23:42</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>93</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>13:23:42</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>96</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>13:23:42</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>104</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>13:23:42</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>107</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>13:23:42</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>15:11</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>108</v>
+      </c>
+      <c r="E170" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4431,7 +4606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4444,14 +4619,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:56:54</t>
+          <t>Última actualización: 13:23:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -4960,7 +5135,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4974,7 +5149,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4985,7 +5160,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4999,7 +5174,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>91</v>
+        <v>64</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -5035,7 +5210,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5049,9 +5224,34 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>111</v>
+        <v>84</v>
       </c>
       <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>13:23:42</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>93</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5068,7 +5268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5081,14 +5281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:56:54</t>
+          <t>Última actualización: 13:23:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5772,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5586,7 +5786,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -5622,7 +5822,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:23:42</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5636,7 +5836,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -5666,6 +5866,56 @@
       <c r="E27" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:23:42</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>64</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>13:23:42</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:12</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>109</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1631
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E170"/>
+  <dimension ref="A1:E177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:23:42</t>
+          <t>Última actualización: 13:53:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 165</t>
+          <t>Total filas: 172</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>14:07</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>71</v>
+        <v>2</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,12 +4148,12 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>14:07</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -4162,7 +4162,7 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,12 +4248,12 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -4262,7 +4262,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>98</v>
+        <v>23</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>62</v>
+        <v>98</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4303,16 +4303,16 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:26</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,12 +4348,12 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -4362,7 +4362,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>109</v>
+        <v>34</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>12:39:18</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,12 +4398,12 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -4412,7 +4412,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>78</v>
+        <v>104</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>84</v>
+        <v>48</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>93</v>
+        <v>62</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>96</v>
+        <v>63</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4528,16 +4528,16 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>107</v>
+        <v>68</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,23 +4573,198 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
+          <t>13:53:48</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>72</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>13:53:48</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>74</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
           <t>13:23:42</t>
         </is>
       </c>
-      <c r="B170" t="inlineStr">
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>107</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>13:53:48</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
         <is>
           <t>15:11</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr">
+      <c r="C173" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D170" t="n">
-        <v>108</v>
-      </c>
-      <c r="E170" t="inlineStr">
+      <c r="D173" t="n">
+        <v>78</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>13:53:48</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>93</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>13:53:48</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>94</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>13:53:48</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>114</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>13:53:48</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>115</v>
+      </c>
+      <c r="E177" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4606,7 +4781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4619,14 +4794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:23:42</t>
+          <t>Última actualización: 13:53:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -5160,7 +5335,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5174,7 +5349,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -5210,7 +5385,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5224,7 +5399,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>84</v>
+        <v>54</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5235,7 +5410,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5249,9 +5424,34 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>93</v>
+        <v>63</v>
       </c>
       <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>13:53:48</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>94</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5268,7 +5468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5281,14 +5481,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:23:42</t>
+          <t>Última actualización: 13:53:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -5872,12 +6072,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -5886,7 +6086,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5897,23 +6097,48 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>34</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>13:53:48</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>15:12</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>109</v>
-      </c>
-      <c r="E29" t="inlineStr">
+      <c r="D30" t="n">
+        <v>79</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1632
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E177"/>
+  <dimension ref="A1:E190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:53:48</t>
+          <t>Última actualización: 14:18:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 172</t>
+          <t>Total filas: 185</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>38</v>
+        <v>67</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:18</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4353,16 +4353,16 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:26</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>109</v>
+        <v>9</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>104</v>
+        <v>34</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>54</v>
+        <v>104</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>62</v>
+        <v>23</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4503,16 +4503,16 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>13:23:42</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>96</v>
+        <v>30</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4578,16 +4578,16 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>14:57</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>74</v>
+        <v>39</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4628,16 +4628,16 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4653,16 +4653,16 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:02</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>93</v>
+        <v>44</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4703,16 +4703,16 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>114</v>
+        <v>49</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,23 +4748,348 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>52</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>15:11</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>53</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
           <t>13:53:48</t>
         </is>
       </c>
-      <c r="B177" t="inlineStr">
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>93</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>69</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>13:53:48</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>94</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>70</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>13:53:48</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>114</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
         <is>
           <t>15:48</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
+      <c r="C184" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D177" t="n">
-        <v>115</v>
-      </c>
-      <c r="E177" t="inlineStr">
+      <c r="D184" t="n">
+        <v>90</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>90</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>97</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>99</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>99</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>109</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>16:08</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>110</v>
+      </c>
+      <c r="E190" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4781,7 +5106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4794,14 +5119,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:53:48</t>
+          <t>Última actualización: 14:18:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5685,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12:39:18</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5374,7 +5699,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>109</v>
+        <v>10</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -5410,21 +5735,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>63</v>
+        <v>30</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5440,18 +5765,93 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>63</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>39</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>13:53:48</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>15:27</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D32" t="n">
         <v>94</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>70</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5468,7 +5868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5481,14 +5881,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:53:48</t>
+          <t>Última actualización: 14:18:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -6122,25 +6522,100 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>10</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>13:53:48</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>15:12</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D31" t="n">
         <v>79</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>15:13</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>55</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>95</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1633
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E190"/>
+  <dimension ref="A1:E201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:18:01</t>
+          <t>Última actualización: 14:46:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 185</t>
+          <t>Total filas: 196</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>38</v>
+        <v>67</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4408,11 +4408,11 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4512,7 +4512,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4548,7 +4548,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -4562,7 +4562,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>63</v>
+        <v>10</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>68</v>
+        <v>15</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4737,7 +4737,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,7 +4748,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -4762,7 +4762,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4787,7 +4787,7 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>93</v>
+        <v>39</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,12 +4823,12 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -4837,7 +4837,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>69</v>
+        <v>40</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>94</v>
+        <v>41</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4878,16 +4878,16 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>114</v>
+        <v>70</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,12 +4948,12 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -4962,7 +4962,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>90</v>
+        <v>114</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>97</v>
+        <v>62</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5003,16 +5003,16 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5028,16 +5028,16 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>109</v>
+        <v>70</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,23 +5073,298 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
+          <t>14:46:40</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>70</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
           <t>14:18:01</t>
         </is>
       </c>
-      <c r="B190" t="inlineStr">
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>99</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>99</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>14:46:40</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>16:01</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>75</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>14:46:40</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>81</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>14:18:01</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
         <is>
           <t>16:08</t>
         </is>
       </c>
-      <c r="C190" t="inlineStr">
+      <c r="C195" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D190" t="n">
+      <c r="D195" t="n">
         <v>110</v>
       </c>
-      <c r="E190" t="inlineStr">
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>14:46:40</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>16:11</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>85</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>14:46:40</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>97</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>14:46:40</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>16:26</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>100</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>14:46:40</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>112</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>14:46:40</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>114</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>14:46:40</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>115</v>
+      </c>
+      <c r="E201" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5119,7 +5394,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:18:01</t>
+          <t>Última actualización: 14:46:40</t>
         </is>
       </c>
     </row>
@@ -5710,7 +5985,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5724,7 +5999,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5760,7 +6035,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5774,7 +6049,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>63</v>
+        <v>10</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5810,7 +6085,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5824,7 +6099,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>94</v>
+        <v>41</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5868,7 +6143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5881,14 +6156,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:18:01</t>
+          <t>Última actualización: 14:46:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -6547,7 +6822,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -6561,7 +6836,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>79</v>
+        <v>26</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -6597,25 +6872,75 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>14:46:40</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>15:52</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>66</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>14:18:01</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>15:53</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D34" t="n">
         <v>95</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>14:46:40</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>16:37</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>111</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1634
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E201"/>
+  <dimension ref="A1:E207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:46:40</t>
+          <t>Última actualización: 15:01:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 196</t>
+          <t>Total filas: 202</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -583,11 +583,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -608,11 +608,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4408,11 +4408,11 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>15:02</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,12 +4698,12 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -4712,7 +4712,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:02</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,12 +4748,12 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -4762,7 +4762,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4803,16 +4803,16 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,12 +4873,12 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>69</v>
+        <v>25</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4903,16 +4903,16 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4928,16 +4928,16 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>114</v>
+        <v>27</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,12 +4998,12 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -5012,7 +5012,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>90</v>
+        <v>114</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>97</v>
+        <v>47</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>70</v>
+        <v>97</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,12 +5098,12 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -5112,7 +5112,7 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>99</v>
+        <v>55</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,12 +5123,12 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>99</v>
+        <v>70</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>16:01</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,21 +5198,21 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>16:08</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>110</v>
+        <v>59</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5228,16 +5228,16 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>16:11</t>
+          <t>16:01</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:07</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>97</v>
+        <v>66</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>16:26</t>
+          <t>16:08</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>112</v>
+        <v>70</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>114</v>
+        <v>82</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,23 +5348,173 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
+          <t>15:01:20</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>16:26</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>85</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>15:01:20</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>89</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>15:01:20</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>97</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
           <t>14:46:40</t>
         </is>
       </c>
-      <c r="B201" t="inlineStr">
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>114</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>15:01:20</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
         <is>
           <t>16:41</t>
         </is>
       </c>
-      <c r="C201" t="inlineStr">
+      <c r="C205" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D201" t="n">
+      <c r="D205" t="n">
+        <v>100</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>15:01:20</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>112</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>15:01:20</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
         <v>115</v>
       </c>
-      <c r="E201" t="inlineStr">
+      <c r="E207" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5394,7 +5544,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:46:40</t>
+          <t>Última actualización: 15:01:20</t>
         </is>
       </c>
     </row>
@@ -6110,7 +6260,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6124,7 +6274,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6143,7 +6293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6156,14 +6306,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:46:40</t>
+          <t>Última actualización: 15:01:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -6847,7 +6997,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -6861,7 +7011,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -6897,7 +7047,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6911,7 +7061,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>95</v>
+        <v>52</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -6939,6 +7089,31 @@
         <v>111</v>
       </c>
       <c r="E35" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>15:01:20</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>97</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1635
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E207"/>
+  <dimension ref="A1:E219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:01:20</t>
+          <t>Última actualización: 15:55:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 202</t>
+          <t>Total filas: 214</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -583,11 +583,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -608,11 +608,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4408,11 +4408,11 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>41</v>
+        <v>69</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>90</v>
+        <v>47</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5153,16 +5153,16 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5183,11 +5183,11 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>99</v>
+        <v>2</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,21 +5198,21 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>59</v>
+        <v>2</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,12 +5223,12 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>16:01</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -5237,7 +5237,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>16:01</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>16:08</t>
+          <t>16:07</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>110</v>
+        <v>12</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,12 +5298,12 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>16:11</t>
+          <t>16:08</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -5312,7 +5312,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>82</v>
+        <v>16</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>16:26</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>85</v>
+        <v>28</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>89</v>
+        <v>30</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5403,16 +5403,16 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:26</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>16:27</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>114</v>
+        <v>32</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:29</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>100</v>
+        <v>34</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5478,16 +5478,16 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>16:53</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,23 +5498,323 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>43</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>45</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>46</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>58</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
           <t>15:01:20</t>
         </is>
       </c>
-      <c r="B207" t="inlineStr">
+      <c r="B211" t="inlineStr">
         <is>
           <t>16:56</t>
         </is>
       </c>
-      <c r="C207" t="inlineStr">
+      <c r="C211" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D207" t="n">
+      <c r="D211" t="n">
         <v>115</v>
       </c>
-      <c r="E207" t="inlineStr">
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>16:57</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>62</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>73</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>87</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>98</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>100</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>102</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>103</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>17:50</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>115</v>
+      </c>
+      <c r="E219" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5531,7 +5831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5544,14 +5844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:01:20</t>
+          <t>Última actualización: 15:55:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -6277,6 +6577,56 @@
         <v>27</v>
       </c>
       <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>73</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>98</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6293,7 +6643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6306,14 +6656,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:01:20</t>
+          <t>Última actualización: 15:55:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -7097,7 +7447,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7111,11 +7461,36 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>17:03</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>68</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1636
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E219"/>
+  <dimension ref="A1:E229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:55:13</t>
+          <t>Última actualización: 16:20:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 214</t>
+          <t>Total filas: 224</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>38</v>
+        <v>67</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4408,11 +4408,11 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>41</v>
+        <v>69</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>90</v>
+        <v>47</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>1</v>
+        <v>55</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:22</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>16:26</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>85</v>
+        <v>5</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,12 +5423,12 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>16:27</t>
+          <t>16:26</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5453,16 +5453,16 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>16:29</t>
+          <t>16:27</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,12 +5473,12 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:29</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>89</v>
+        <v>34</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,21 +5498,21 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>16:38</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:40</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>16:53</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>115</v>
+        <v>21</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>16:57</t>
+          <t>16:53</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>73</v>
+        <v>35</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>87</v>
+        <v>36</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5703,16 +5703,16 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>16:57</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>98</v>
+        <v>62</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,21 +5748,21 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:16</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>102</v>
+        <v>56</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,21 +5773,21 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>103</v>
+        <v>62</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,23 +5798,273 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
+          <t>16:20:28</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>72</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
           <t>15:55:13</t>
         </is>
       </c>
-      <c r="B219" t="inlineStr">
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>98</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>100</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>16:20:28</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>76</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>15:55:13</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>102</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>16:20:28</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>78</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>16:20:28</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>17:43</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>83</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>16:20:28</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
         <is>
           <t>17:50</t>
         </is>
       </c>
-      <c r="C219" t="inlineStr">
+      <c r="C226" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D219" t="n">
-        <v>115</v>
-      </c>
-      <c r="E219" t="inlineStr">
+      <c r="D226" t="n">
+        <v>90</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>16:20:28</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>93</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>16:20:28</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>105</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>16:20:28</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>108</v>
+      </c>
+      <c r="E229" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5831,7 +6081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5844,14 +6094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:55:13</t>
+          <t>Última actualización: 16:20:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -6585,7 +6835,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6599,7 +6849,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>73</v>
+        <v>48</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -6610,23 +6860,73 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>16:20:28</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>72</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>15:55:13</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>17:33</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D35" t="n">
+      <c r="D36" t="n">
         <v>98</v>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>16:20:28</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>93</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6656,7 +6956,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:55:13</t>
+          <t>Última actualización: 16:20:28</t>
         </is>
       </c>
     </row>
@@ -7447,7 +7747,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7461,7 +7761,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -7472,7 +7772,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7486,7 +7786,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1637
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E229"/>
+  <dimension ref="A1:E239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:20:28</t>
+          <t>Última actualización: 16:47:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 224</t>
+          <t>Total filas: 234</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4408,11 +4408,11 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>1</v>
+        <v>55</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>16:53</t>
+          <t>16:47</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:47</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:53</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>16:57</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>62</v>
+        <v>8</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5728,16 +5728,16 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,21 +5748,21 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>17:16</t>
+          <t>16:57</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>56</v>
+        <v>10</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,21 +5773,21 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5803,16 +5803,16 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:16</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>98</v>
+        <v>35</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5878,16 +5878,16 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>102</v>
+        <v>46</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>78</v>
+        <v>100</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5953,16 +5953,16 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>17:43</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>105</v>
+        <v>53</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6053,18 +6053,268 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
+          <t>17:43</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>83</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>16:47:03</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>17:50</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>63</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>16:47:03</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>66</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>16:20:28</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>105</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>16:47:03</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>18:06</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>79</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>16:47:03</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
           <t>18:08</t>
         </is>
       </c>
-      <c r="C229" t="inlineStr">
+      <c r="C234" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D229" t="n">
-        <v>108</v>
-      </c>
-      <c r="E229" t="inlineStr">
+      <c r="D234" t="n">
+        <v>81</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>16:47:03</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>93</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>16:47:03</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>95</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>16:47:03</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>96</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>16:47:03</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>109</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>16:47:03</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>110</v>
+      </c>
+      <c r="E239" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6081,7 +6331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6094,14 +6344,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:20:28</t>
+          <t>Última actualización: 16:47:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -6835,7 +7085,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6849,7 +7099,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -6885,7 +7135,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6899,7 +7149,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>98</v>
+        <v>46</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6910,7 +7160,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6924,9 +7174,34 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>93</v>
+        <v>66</v>
       </c>
       <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>16:47:03</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>96</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6943,7 +7218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6956,14 +7231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:20:28</t>
+          <t>Última actualización: 16:47:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -7772,7 +8047,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7786,9 +8061,34 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="E37" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>16:47:03</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>103</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1638
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E239"/>
+  <dimension ref="A1:E246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:47:03</t>
+          <t>Última actualización: 16:59:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 234</t>
+          <t>Total filas: 241</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -583,11 +583,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -608,11 +608,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>41</v>
+        <v>69</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5773,21 +5773,21 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>17:16</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>56</v>
+        <v>9</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:16</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>17:25</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>100</v>
+        <v>33</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>76</v>
+        <v>46</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6028,16 +6028,16 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>17:43</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6078,16 +6078,16 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:43</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>18:06</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6203,16 +6203,16 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:06</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6278,16 +6278,16 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>109</v>
+        <v>95</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,23 +6298,198 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
+          <t>16:59:32</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>84</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>16:59:32</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>86</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>16:59:32</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>18:26</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>87</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>16:59:32</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>96</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
           <t>16:47:03</t>
         </is>
       </c>
-      <c r="B239" t="inlineStr">
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>109</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>16:59:32</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
         <is>
           <t>18:37</t>
         </is>
       </c>
-      <c r="C239" t="inlineStr">
+      <c r="C244" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D239" t="n">
-        <v>110</v>
-      </c>
-      <c r="E239" t="inlineStr">
+      <c r="D244" t="n">
+        <v>98</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>16:59:32</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>18:50</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>111</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>16:59:32</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>114</v>
+      </c>
+      <c r="E246" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6344,7 +6519,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:47:03</t>
+          <t>Última actualización: 16:59:32</t>
         </is>
       </c>
     </row>
@@ -7085,7 +7260,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7099,7 +7274,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -7110,7 +7285,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7124,7 +7299,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -7160,7 +7335,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7174,7 +7349,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -7185,7 +7360,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7199,7 +7374,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -7231,7 +7406,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:47:03</t>
+          <t>Última actualización: 16:59:32</t>
         </is>
       </c>
     </row>
@@ -8047,7 +8222,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -8061,7 +8236,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -8072,7 +8247,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -8086,7 +8261,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1639
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E246"/>
+  <dimension ref="A1:E256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:59:32</t>
+          <t>Última actualización: 17:30:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 241</t>
+          <t>Total filas: 251</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -583,11 +583,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -608,11 +608,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4908,11 +4908,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>41</v>
+        <v>69</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4933,11 +4933,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>1</v>
+        <v>55</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5937,7 +5937,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,7 +5948,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -5958,11 +5958,11 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>100</v>
+        <v>46</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>37</v>
+        <v>100</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,12 +6023,12 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -6037,7 +6037,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>53</v>
+        <v>8</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,12 +6098,12 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>16:20:28</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>17:43</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -6112,7 +6112,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>83</v>
+        <v>53</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:20:28</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:43</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,12 +6198,12 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>18:06</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -6212,7 +6212,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>79</v>
+        <v>35</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>18:06</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>81</v>
+        <v>38</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>95</v>
+        <v>40</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>18:26</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>87</v>
+        <v>53</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>96</v>
+        <v>53</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>109</v>
+        <v>86</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6428,16 +6428,16 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:26</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>18:27</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>111</v>
+        <v>57</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,23 +6473,273 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>65</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>16:47:03</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>109</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>67</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>18:50</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>80</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
           <t>18:53</t>
         </is>
       </c>
-      <c r="C246" t="inlineStr">
+      <c r="C250" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D246" t="n">
-        <v>114</v>
-      </c>
-      <c r="E246" t="inlineStr">
+      <c r="D250" t="n">
+        <v>83</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>85</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>95</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>98</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>106</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>111</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>113</v>
+      </c>
+      <c r="E256" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6506,7 +6756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6519,14 +6769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:59:32</t>
+          <t>Última actualización: 17:30:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -7285,7 +7535,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7299,7 +7549,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -7335,7 +7585,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7349,7 +7599,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -7360,7 +7610,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7374,9 +7624,59 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>84</v>
+        <v>53</v>
       </c>
       <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>98</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>113</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7393,7 +7693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7406,14 +7706,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:59:32</t>
+          <t>Última actualización: 17:30:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -8247,25 +8547,75 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>18:29</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>59</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>16:59:32</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D39" t="n">
         <v>91</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>19:02</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>92</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1640
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E256"/>
+  <dimension ref="A1:E267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:30:34</t>
+          <t>Última actualización: 17:56:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 251</t>
+          <t>Total filas: 262</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -583,11 +583,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -608,11 +608,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>90</v>
+        <v>47</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6212,7 +6212,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6248,7 +6248,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -6262,7 +6262,7 @@
         </is>
       </c>
       <c r="D237" t="n">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,7 +6273,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -6287,7 +6287,7 @@
         </is>
       </c>
       <c r="D238" t="n">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,12 +6298,12 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:19</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -6312,7 +6312,7 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>95</v>
+        <v>50</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,12 +6348,12 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -6362,7 +6362,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,21 +6423,21 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>18:26</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>87</v>
+        <v>53</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>18:27</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:26</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>65</v>
+        <v>87</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,21 +6498,21 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:27</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>109</v>
+        <v>57</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,21 +6523,21 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,21 +6548,21 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>83</v>
+        <v>41</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,21 +6598,21 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:49</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6628,16 +6628,16 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:50</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>98</v>
+        <v>57</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,21 +6673,21 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>106</v>
+        <v>59</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,21 +6698,21 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>111</v>
+        <v>68</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6728,18 +6728,293 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>95</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>17:56:52</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>19:07</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>71</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>98</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>17:56:52</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>19:13</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>77</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>106</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>17:56:52</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>85</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>17:56:52</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>86</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>17:56:52</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>86</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
           <t>19:23</t>
         </is>
       </c>
-      <c r="C256" t="inlineStr">
+      <c r="C264" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D256" t="n">
+      <c r="D264" t="n">
         <v>113</v>
       </c>
-      <c r="E256" t="inlineStr">
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>17:56:52</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>104</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>17:56:52</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>104</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>17:56:52</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>107</v>
+      </c>
+      <c r="E267" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6756,7 +7031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6769,14 +7044,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:30:34</t>
+          <t>Última actualización: 17:56:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -7610,12 +7885,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -7624,7 +7899,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -7640,16 +7915,16 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -7660,23 +7935,98 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>17:56:52</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>19:07</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>71</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>17:30:34</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>98</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>17:56:52</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>86</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>17:30:34</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
         <is>
           <t>19:23</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D40" t="n">
+      <c r="D43" t="n">
         <v>113</v>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7693,7 +8043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7706,14 +8056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:30:34</t>
+          <t>Última actualización: 17:56:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -8547,7 +8897,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -8561,7 +8911,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -8597,23 +8947,48 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>17:56:52</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>19:01</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>65</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>17:30:34</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>19:02</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D40" t="n">
+      <c r="D41" t="n">
         <v>92</v>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1641
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E267"/>
+  <dimension ref="A1:E273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:56:52</t>
+          <t>Última actualización: 18:21:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 262</t>
+          <t>Total filas: 268</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:30:32</t>
+          <t>03:38:59</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -583,11 +583,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:38:59</t>
+          <t>04:30:32</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -608,11 +608,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>38</v>
+        <v>67</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -6348,12 +6348,12 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -6362,7 +6362,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,12 +6373,12 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -6387,7 +6387,7 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,21 +6423,21 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>16:59:32</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>18:26</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>87</v>
+        <v>53</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,21 +6498,21 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>18:27</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,21 +6523,21 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,21 +6548,21 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>16:59:32</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:26</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>109</v>
+        <v>87</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:27</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,21 +6598,21 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>18:49</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,21 +6623,21 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6678,16 +6678,16 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:49</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,21 +6698,21 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>18:50</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,21 +6723,21 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>95</v>
+        <v>32</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,21 +6748,21 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>19:07</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>71</v>
+        <v>34</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,21 +6773,21 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>98</v>
+        <v>68</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6798,21 +6798,21 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>19:13</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,21 +6823,21 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,21 +6848,21 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>85</v>
+        <v>47</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6878,16 +6878,16 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:13</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,21 +6898,21 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,21 +6923,21 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>113</v>
+        <v>60</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6953,16 +6953,16 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6978,16 +6978,16 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,23 +6998,173 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
+          <t>18:21:35</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>62</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>18:21:35</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>19:28</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>67</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
           <t>17:56:52</t>
         </is>
       </c>
-      <c r="B267" t="inlineStr">
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>104</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>18:21:35</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>79</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>18:21:35</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>19:41</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>80</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>18:21:35</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
         <is>
           <t>19:43</t>
         </is>
       </c>
-      <c r="C267" t="inlineStr">
+      <c r="C272" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D267" t="n">
-        <v>107</v>
-      </c>
-      <c r="E267" t="inlineStr">
+      <c r="D272" t="n">
+        <v>82</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>18:21:35</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>101</v>
+      </c>
+      <c r="E273" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7031,7 +7181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7044,14 +7194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:56:52</t>
+          <t>Última actualización: 18:21:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -7885,12 +8035,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -7899,7 +8049,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -7910,12 +8060,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -7924,7 +8074,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -7935,21 +8085,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>19:07</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -7960,12 +8110,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -7974,7 +8124,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>98</v>
+        <v>71</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -7985,21 +8135,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>86</v>
+        <v>47</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8010,23 +8160,48 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>86</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>18:21:35</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>19:23</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>113</v>
-      </c>
-      <c r="E43" t="inlineStr">
+      <c r="D44" t="n">
+        <v>62</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8043,7 +8218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8056,14 +8231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:56:52</t>
+          <t>Última actualización: 18:21:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -8897,7 +9072,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -8911,7 +9086,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -8972,7 +9147,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8986,11 +9161,36 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>92</v>
+        <v>41</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>18:21:35</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>100</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1642
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E273"/>
+  <dimension ref="A1:E283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:21:35</t>
+          <t>Última actualización: 18:47:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 268</t>
+          <t>Total filas: 278</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4408,11 +4408,11 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>1</v>
+        <v>55</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6508,7 +6508,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -6723,21 +6723,21 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,21 +6748,21 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,21 +6773,21 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6798,12 +6798,12 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -6812,7 +6812,7 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,21 +6823,21 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>19:07</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>71</v>
+        <v>18</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,12 +6848,12 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -6862,7 +6862,7 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,21 +6873,21 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>19:13</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>77</v>
+        <v>47</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,21 +6898,21 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,21 +6923,21 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:13</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,21 +6948,21 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,21 +6973,21 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>86</v>
+        <v>34</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,21 +6998,21 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,21 +7023,21 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>19:28</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>67</v>
+        <v>35</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,21 +7048,21 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,21 +7073,21 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>79</v>
+        <v>38</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7103,16 +7103,16 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:28</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,21 +7123,21 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>82</v>
+        <v>53</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,23 +7148,273 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>104</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>18:47:38</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>19:41</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>54</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>18:47:38</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>56</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>18:47:38</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>19:57</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>70</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>18:47:38</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>74</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>18:47:38</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
           <t>20:02</t>
         </is>
       </c>
-      <c r="C273" t="inlineStr">
+      <c r="C278" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D273" t="n">
-        <v>101</v>
-      </c>
-      <c r="E273" t="inlineStr">
+      <c r="D278" t="n">
+        <v>75</v>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>18:47:38</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>75</v>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>18:47:38</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>95</v>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>18:47:38</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>20:25</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>98</v>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>18:47:38</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>114</v>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>18:47:38</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>118</v>
+      </c>
+      <c r="E283" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7181,7 +7431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7194,14 +7444,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:21:35</t>
+          <t>Última actualización: 18:47:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -8110,7 +8360,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8124,7 +8374,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -8160,7 +8410,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -8174,7 +8424,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>86</v>
+        <v>35</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -8202,6 +8452,56 @@
         <v>62</v>
       </c>
       <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>18:47:38</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>75</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>18:47:38</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>114</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8218,7 +8518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8231,14 +8531,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:21:35</t>
+          <t>Última actualización: 18:47:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -9147,7 +9447,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -9161,7 +9461,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -9172,7 +9472,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -9186,9 +9486,34 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>100</v>
+        <v>74</v>
       </c>
       <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>18:47:38</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>114</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1643
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E283"/>
+  <dimension ref="A1:E288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:47:38</t>
+          <t>Última actualización: 19:00:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 278</t>
+          <t>Total filas: 283</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4408,11 +4408,11 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6823,7 +6823,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -6837,7 +6837,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6887,7 +6887,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -6912,7 +6912,7 @@
         </is>
       </c>
       <c r="D263" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6973,21 +6973,21 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,21 +6998,21 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>86</v>
+        <v>21</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,7 +7023,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -7033,11 +7033,11 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>35</v>
+        <v>86</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,12 +7048,12 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -7062,7 +7062,7 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>62</v>
+        <v>35</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,21 +7073,21 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,21 +7098,21 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>19:28</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,21 +7123,21 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:27</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,21 +7148,21 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:21:35</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:28</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>104</v>
+        <v>67</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,12 +7173,12 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -7187,7 +7187,7 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>54</v>
+        <v>104</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,21 +7198,21 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,21 +7223,21 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>19:57</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,21 +7248,21 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>74</v>
+        <v>43</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>19:57</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,21 +7298,21 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7328,16 +7328,16 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>98</v>
+        <v>62</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,21 +7373,21 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>114</v>
+        <v>63</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7403,18 +7403,143 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>95</v>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>19:00:20</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>83</v>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>19:00:20</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>20:25</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>85</v>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>19:00:20</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>101</v>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>19:00:20</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
           <t>20:45</t>
         </is>
       </c>
-      <c r="C283" t="inlineStr">
+      <c r="C287" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D283" t="n">
-        <v>118</v>
-      </c>
-      <c r="E283" t="inlineStr">
+      <c r="D287" t="n">
+        <v>105</v>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>19:00:20</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>117</v>
+      </c>
+      <c r="E288" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7431,7 +7556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7444,14 +7569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:47:38</t>
+          <t>Última actualización: 19:00:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 42</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8510,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8399,7 +8524,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8435,7 +8560,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:21:35</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8449,7 +8574,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>62</v>
+        <v>23</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -8485,23 +8610,48 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>20:03</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>63</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>19:00:20</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D46" t="n">
-        <v>114</v>
-      </c>
-      <c r="E46" t="inlineStr">
+      <c r="D47" t="n">
+        <v>101</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8518,7 +8668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8531,14 +8681,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:47:38</t>
+          <t>Última actualización: 19:00:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -9447,7 +9597,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:00:20</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -9461,7 +9611,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -9497,23 +9647,73 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>19:00:20</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>62</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>18:47:38</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D43" t="n">
+      <c r="D44" t="n">
         <v>114</v>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>19:00:20</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>102</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1644
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E288"/>
+  <dimension ref="A1:E295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:00:20</t>
+          <t>Última actualización: 19:31:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 283</t>
+          <t>Total filas: 290</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>38</v>
+        <v>67</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5948,7 +5948,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -5958,11 +5958,11 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>3</v>
+        <v>46</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5983,11 +5983,11 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -7198,7 +7198,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>19:00:20</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -7212,7 +7212,7 @@
         </is>
       </c>
       <c r="D275" t="n">
-        <v>40</v>
+        <v>9</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,7 +7223,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>19:00:20</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -7237,7 +7237,7 @@
         </is>
       </c>
       <c r="D276" t="n">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,7 +7248,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>19:00:20</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
@@ -7262,7 +7262,7 @@
         </is>
       </c>
       <c r="D277" t="n">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,12 +7273,12 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>19:00:20</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>19:57</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -7287,7 +7287,7 @@
         </is>
       </c>
       <c r="D278" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7303,16 +7303,16 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:57</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,21 +7323,21 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>19:00:20</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,21 +7373,21 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>19:00:20</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>20:03</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,21 +7398,21 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>95</v>
+        <v>32</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,12 +7423,12 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>19:00:20</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:22</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -7437,7 +7437,7 @@
         </is>
       </c>
       <c r="D284" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,21 +7448,21 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>19:00:20</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>85</v>
+        <v>52</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,21 +7473,21 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>19:00:20</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:25</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>101</v>
+        <v>54</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,21 +7498,21 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>19:00:20</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,23 +7523,198 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
+          <t>19:31:25</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>74</v>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>19:31:25</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>80</v>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>19:31:25</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>20:53</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>82</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>19:31:25</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>20:54</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>83</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
           <t>19:00:20</t>
         </is>
       </c>
-      <c r="B288" t="inlineStr">
+      <c r="B292" t="inlineStr">
         <is>
           <t>20:57</t>
         </is>
       </c>
-      <c r="C288" t="inlineStr">
+      <c r="C292" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D288" t="n">
+      <c r="D292" t="n">
         <v>117</v>
       </c>
-      <c r="E288" t="inlineStr">
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>19:31:25</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>92</v>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>19:31:25</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>21:10</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>99</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>19:31:25</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>115</v>
+      </c>
+      <c r="E295" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7569,7 +7744,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:00:20</t>
+          <t>Última actualización: 19:31:25</t>
         </is>
       </c>
     </row>
@@ -8610,7 +8785,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>19:00:20</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8624,7 +8799,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -8635,7 +8810,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>19:00:20</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8649,7 +8824,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>101</v>
+        <v>70</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -8681,7 +8856,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:00:20</t>
+          <t>Última actualización: 19:31:25</t>
         </is>
       </c>
     </row>
@@ -9647,7 +9822,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>19:00:20</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -9661,7 +9836,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -9697,7 +9872,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>19:00:20</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -9711,7 +9886,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>102</v>
+        <v>71</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1645
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E295"/>
+  <dimension ref="A1:E302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:31:25</t>
+          <t>Última actualización: 19:58:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 290</t>
+          <t>Total filas: 297</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>38</v>
+        <v>67</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:43:13</t>
+          <t>12:56:54</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:56:54</t>
+          <t>11:43:13</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6508,7 +6508,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -7023,7 +7023,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -7033,11 +7033,11 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>86</v>
+        <v>35</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,7 +7048,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -7058,11 +7058,11 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>35</v>
+        <v>86</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7398,7 +7398,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>19:58:17</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -7408,11 +7408,11 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:58:17</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>95</v>
+        <v>5</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,21 +7448,21 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>19:58:17</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:08</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,21 +7473,21 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:22</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>54</v>
+        <v>95</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,21 +7498,21 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>19:58:17</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,21 +7523,21 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>19:58:17</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:25</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,21 +7548,21 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>19:58:17</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:37</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>80</v>
+        <v>39</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7578,16 +7578,16 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>20:53</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,21 +7598,21 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>19:58:17</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>20:54</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>83</v>
+        <v>44</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7623,21 +7623,21 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>19:00:20</t>
+          <t>19:58:17</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>117</v>
+        <v>47</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,21 +7648,21 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>19:58:17</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>92</v>
+        <v>53</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7678,16 +7678,16 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>20:53</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7703,18 +7703,193 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
+          <t>20:54</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>83</v>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>19:58:17</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>59</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>19:58:17</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>65</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>19:58:17</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>21:10</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>72</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>19:58:17</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
           <t>21:26</t>
         </is>
       </c>
-      <c r="C295" t="inlineStr">
+      <c r="C299" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D295" t="n">
-        <v>115</v>
-      </c>
-      <c r="E295" t="inlineStr">
+      <c r="D299" t="n">
+        <v>88</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>19:58:17</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>96</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>19:58:17</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>21:39</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>101</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>19:58:17</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>21:46</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>108</v>
+      </c>
+      <c r="E302" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7731,7 +7906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7744,14 +7919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:31:25</t>
+          <t>Última actualización: 19:58:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 42</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -8785,7 +8960,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>19:58:17</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8799,7 +8974,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -8827,6 +9002,31 @@
         <v>70</v>
       </c>
       <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>19:58:17</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>44</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8843,7 +9043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8856,14 +9056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:31:25</t>
+          <t>Última actualización: 19:58:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -9797,12 +9997,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:58:17</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:58</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -9811,7 +10011,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -9822,12 +10022,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -9836,7 +10036,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>31</v>
+        <v>74</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -9847,12 +10047,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -9861,7 +10061,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>114</v>
+        <v>31</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -9872,23 +10072,48 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>114</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>19:58:17</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
           <t>20:42</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D45" t="n">
-        <v>71</v>
-      </c>
-      <c r="E45" t="inlineStr">
+      <c r="D46" t="n">
+        <v>44</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1646
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E302"/>
+  <dimension ref="A1:E309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:58:17</t>
+          <t>Última actualización: 20:26:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 297</t>
+          <t>Total filas: 304</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>90</v>
+        <v>47</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>15:01:20</t>
+          <t>15:55:13</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>14:46:40</t>
+          <t>15:01:20</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>15:55:13</t>
+          <t>14:46:40</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5948,7 +5948,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -5958,11 +5958,11 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5983,11 +5983,11 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>3</v>
+        <v>46</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6508,7 +6508,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -7348,7 +7348,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>75</v>
+        <v>31</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,7 +7373,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -7383,11 +7383,11 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>31</v>
+        <v>75</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7573,7 +7573,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>20:26:22</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -7587,7 +7587,7 @@
         </is>
       </c>
       <c r="D290" t="n">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,21 +7598,21 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>19:58:17</t>
+          <t>20:26:22</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7628,16 +7628,16 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,21 +7648,21 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>19:58:17</t>
+          <t>20:26:22</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,21 +7673,21 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>20:26:22</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>20:53</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,21 +7698,21 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>19:58:17</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>20:54</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>83</v>
+        <v>53</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,21 +7723,21 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>19:58:17</t>
+          <t>20:26:22</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:52</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>59</v>
+        <v>26</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,21 +7748,21 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>19:58:17</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>20:53</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,21 +7773,21 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>19:58:17</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>20:54</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>19:58:17</t>
+          <t>20:26:22</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>88</v>
+        <v>31</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,21 +7823,21 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>19:58:17</t>
+          <t>20:26:22</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:03</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>96</v>
+        <v>37</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7853,16 +7853,16 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>21:39</t>
+          <t>21:10</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>101</v>
+        <v>72</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -7873,23 +7873,198 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
+          <t>20:26:22</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>60</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>20:26:22</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>68</v>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
           <t>19:58:17</t>
         </is>
       </c>
-      <c r="B302" t="inlineStr">
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>21:39</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>101</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>20:26:22</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
         <is>
           <t>21:46</t>
         </is>
       </c>
-      <c r="C302" t="inlineStr">
+      <c r="C305" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D302" t="n">
-        <v>108</v>
-      </c>
-      <c r="E302" t="inlineStr">
+      <c r="D305" t="n">
+        <v>80</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>20:26:22</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>83</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>20:26:22</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>22:04</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>98</v>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>20:26:22</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>22:13</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D308" t="n">
+        <v>107</v>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>20:26:22</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>22:22</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>116</v>
+      </c>
+      <c r="E309" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7919,7 +8094,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:58:17</t>
+          <t>Última actualización: 20:26:22</t>
         </is>
       </c>
     </row>
@@ -8985,7 +9160,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>20:26:22</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8999,7 +9174,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -9043,7 +9218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9056,14 +9231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:58:17</t>
+          <t>Última actualización: 20:26:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -10097,7 +10272,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>19:58:17</t>
+          <t>20:26:22</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -10111,11 +10286,61 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>20:26:22</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>21:27</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>61</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>20:26:22</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>22:16</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>110</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1647
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E309"/>
+  <dimension ref="A1:E319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:26:22</t>
+          <t>Última actualización: 20:49:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 304</t>
+          <t>Total filas: 314</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:41:47</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:41:47</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>38</v>
+        <v>67</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>13:53:48</t>
+          <t>14:18:01</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>14:18:01</t>
+          <t>13:53:48</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4408,11 +4408,11 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5948,7 +5948,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -5958,11 +5958,11 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>3</v>
+        <v>46</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5983,11 +5983,11 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -7173,7 +7173,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -7183,11 +7183,11 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>104</v>
+        <v>9</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,7 +7198,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -7208,11 +7208,11 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>9</v>
+        <v>104</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>18:47:38</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>31</v>
+        <v>75</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,7 +7373,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>18:47:38</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -7383,11 +7383,11 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>75</v>
+        <v>31</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7408,7 +7408,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D283" t="n">
@@ -7433,7 +7433,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D284" t="n">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -7698,21 +7698,21 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>19:58:17</t>
+          <t>20:49:46</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:50</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,12 +7723,12 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>20:26:22</t>
+          <t>20:49:46</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>20:52</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -7737,7 +7737,7 @@
         </is>
       </c>
       <c r="D296" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,21 +7748,21 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>20:26:22</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>20:53</t>
+          <t>20:52</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>82</v>
+        <v>26</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7778,16 +7778,16 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>20:54</t>
+          <t>20:53</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,12 +7798,12 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>20:26:22</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:54</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -7812,7 +7812,7 @@
         </is>
       </c>
       <c r="D299" t="n">
-        <v>31</v>
+        <v>83</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,21 +7823,21 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>20:26:22</t>
+          <t>20:49:46</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,21 +7848,21 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>19:58:17</t>
+          <t>20:26:22</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>72</v>
+        <v>31</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -7873,21 +7873,21 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>20:26:22</t>
+          <t>20:49:46</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>60</v>
+        <v>13</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -7903,16 +7903,16 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:03</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7928,16 +7928,16 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>21:39</t>
+          <t>21:10</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>101</v>
+        <v>72</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -7948,21 +7948,21 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>20:26:22</t>
+          <t>20:49:46</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>21:46</t>
+          <t>21:26</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>80</v>
+        <v>37</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,21 +7973,21 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>20:26:22</t>
+          <t>20:49:46</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>21:33</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>83</v>
+        <v>44</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -8003,16 +8003,16 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>22:04</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>98</v>
+        <v>68</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,21 +8023,21 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>20:26:22</t>
+          <t>19:58:17</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>22:13</t>
+          <t>21:39</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,23 +8048,273 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
+          <t>20:49:46</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>51</v>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>20:49:46</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>56</v>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
           <t>20:26:22</t>
         </is>
       </c>
-      <c r="B309" t="inlineStr">
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>21:46</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D311" t="n">
+        <v>80</v>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>20:26:22</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>83</v>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>20:49:46</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>22:03</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D313" t="n">
+        <v>74</v>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>20:26:22</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>22:04</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D314" t="n">
+        <v>98</v>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>20:49:46</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D315" t="n">
+        <v>83</v>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>20:49:46</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>22:13</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D316" t="n">
+        <v>84</v>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>20:26:22</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
         <is>
           <t>22:22</t>
         </is>
       </c>
-      <c r="C309" t="inlineStr">
+      <c r="C317" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D309" t="n">
+      <c r="D317" t="n">
         <v>116</v>
       </c>
-      <c r="E309" t="inlineStr">
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>20:49:46</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>104</v>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>20:49:46</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>22:43</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>114</v>
+      </c>
+      <c r="E319" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8081,7 +8331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8094,14 +8344,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:26:22</t>
+          <t>Última actualización: 20:49:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -9202,6 +9452,31 @@
         <v>44</v>
       </c>
       <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>20:49:46</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>104</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9218,7 +9493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9231,14 +9506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:26:22</t>
+          <t>Última actualización: 20:49:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 45</t>
         </is>
       </c>
     </row>
@@ -10322,23 +10597,73 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>20:49:46</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>21:28</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>39</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>20:49:46</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>86</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>20:26:22</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>22:16</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D48" t="n">
+      <c r="D50" t="n">
         <v>110</v>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1648
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-15.xlsx
+++ b/data/horarios-141-2026-03-15.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E319"/>
+  <dimension ref="A1:E326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:49:46</t>
+          <t>Última actualización: 21:03:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 314</t>
+          <t>Total filas: 321</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:54:35</t>
+          <t>07:18:31</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:18:31</t>
+          <t>06:54:35</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:57:38</t>
+          <t>08:16:18</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:16:18</t>
+          <t>08:57:38</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2083,11 +2083,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>09:40:26</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>09:40:26</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>10:35:48</t>
+          <t>11:04:33</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3108,11 +3108,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>11:04:33</t>
+          <t>10:35:48</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>38</v>
+        <v>67</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -5948,7 +5948,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>16:47:03</t>
+          <t>17:30:34</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -5958,11 +5958,11 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>17:30:34</t>
+          <t>16:47:03</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5983,11 +5983,11 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>3</v>
+        <v>46</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6508,7 +6508,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -7173,7 +7173,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>19:31:25</t>
+          <t>17:56:52</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -7183,11 +7183,11 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>9</v>
+        <v>104</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,7 +7198,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>17:56:52</t>
+          <t>19:31:25</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -7208,11 +7208,11 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>104</v>
+        <v>9</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7408,7 +7408,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D283" t="n">
@@ -7433,7 +7433,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D284" t="n">
@@ -7898,7 +7898,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>20:26:22</t>
+          <t>21:03:14</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
@@ -7912,7 +7912,7 @@
         </is>
       </c>
       <c r="D303" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7923,21 +7923,21 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>19:58:17</t>
+          <t>21:03:14</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>21:03</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -7948,21 +7948,21 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>20:49:46</t>
+          <t>19:58:17</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>21:10</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,21 +7973,21 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>20:49:46</t>
+          <t>21:03:14</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>21:33</t>
+          <t>21:26</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -7998,12 +7998,12 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>20:26:22</t>
+          <t>20:49:46</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:33</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -8012,7 +8012,7 @@
         </is>
       </c>
       <c r="D307" t="n">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,21 +8023,21 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>19:58:17</t>
+          <t>21:03:14</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>21:39</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>101</v>
+        <v>31</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,21 +8048,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>20:49:46</t>
+          <t>21:03:14</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>21:40</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8073,21 +8073,21 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>20:49:46</t>
+          <t>19:58:17</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>21:39</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8098,21 +8098,21 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>20:26:22</t>
+          <t>21:03:14</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>21:46</t>
+          <t>21:40</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>80</v>
+        <v>37</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,21 +8123,21 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>20:26:22</t>
+          <t>20:49:46</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,21 +8148,21 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>20:49:46</t>
+          <t>21:03:14</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>22:03</t>
+          <t>21:46</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>74</v>
+        <v>43</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8178,16 +8178,16 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>22:04</t>
+          <t>21:49</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8203,16 +8203,16 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>22:12</t>
+          <t>22:03</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8223,12 +8223,12 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>20:49:46</t>
+          <t>21:03:14</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>22:13</t>
+          <t>22:04</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -8237,7 +8237,7 @@
         </is>
       </c>
       <c r="D316" t="n">
-        <v>84</v>
+        <v>61</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -8248,12 +8248,12 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>20:26:22</t>
+          <t>20:49:46</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>22:22</t>
+          <t>22:12</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -8262,7 +8262,7 @@
         </is>
       </c>
       <c r="D317" t="n">
-        <v>116</v>
+        <v>83</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -8278,16 +8278,16 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>22:33</t>
+          <t>22:13</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>104</v>
+        <v>84</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -8298,23 +8298,198 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
+          <t>21:03:14</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>22:18</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>75</v>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>20:26:22</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>22:22</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D320" t="n">
+        <v>116</v>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>21:03:14</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>22:25</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>82</v>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>21:03:14</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>22:28</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D322" t="n">
+        <v>85</v>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
           <t>20:49:46</t>
         </is>
       </c>
-      <c r="B319" t="inlineStr">
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D323" t="n">
+        <v>104</v>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>21:03:14</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>22:34</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D324" t="n">
+        <v>91</v>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>20:49:46</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
         <is>
           <t>22:43</t>
         </is>
       </c>
-      <c r="C319" t="inlineStr">
+      <c r="C325" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D319" t="n">
+      <c r="D325" t="n">
         <v>114</v>
       </c>
-      <c r="E319" t="inlineStr">
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>21:03:14</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>22:44</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D326" t="n">
+        <v>101</v>
+      </c>
+      <c r="E326" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8331,7 +8506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8344,14 +8519,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:49:46</t>
+          <t>Última actualización: 21:03:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 44</t>
+          <t>Total filas: 45</t>
         </is>
       </c>
     </row>
@@ -9477,6 +9652,31 @@
         <v>104</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>21:03:14</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>22:34</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>91</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9493,7 +9693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9506,14 +9706,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:49:46</t>
+          <t>Última actualización: 21:03:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 45</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -10622,48 +10822,73 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>20:49:46</t>
+          <t>21:03:14</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>22:15</t>
+          <t>21:32</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-40 Y 115</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>20:26:22</t>
+          <t>20:49:46</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>86</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>21:03:14</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
           <t>22:16</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D50" t="n">
-        <v>110</v>
-      </c>
-      <c r="E50" t="inlineStr">
+      <c r="D51" t="n">
+        <v>73</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>